<commit_message>
relatorio excel dia 12-05-26
</commit_message>
<xml_diff>
--- a/saida_skus/SKU_BRINQ-019-VASSOURA-INFANTIL-UNICORNIO.xlsx
+++ b/saida_skus/SKU_BRINQ-019-VASSOURA-INFANTIL-UNICORNIO.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Analise" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analise'!$A$1:$O$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analise'!$A$1:$O$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O83"/>
+  <dimension ref="A1:O85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -559,12 +559,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>12/05/2026</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
           <t>11/05/2026</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>10/05/2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -632,12 +632,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>12/05/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
           <t>11/05/2026</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>10/05/2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -709,14 +709,14 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>11/05/2026</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
           <t>10/05/2026</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>09/05/2026</t>
-        </is>
-      </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -739,7 +739,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -747,10 +747,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I4" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -759,39 +757,37 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Boa</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>11/05/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
           <t>10/05/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -863,12 +859,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
           <t>09/05/2026</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>08/05/2026</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -940,12 +936,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
           <t>09/05/2026</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>08/05/2026</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1017,14 +1013,14 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
           <t>08/05/2026</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -1047,7 +1043,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1055,8 +1051,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I8" s="2" t="n">
-        <v>0</v>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -1065,37 +1063,39 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
           <t>08/05/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1167,12 +1167,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
           <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1240,12 +1240,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
           <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1317,12 +1317,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
           <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>05/05/2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1390,12 +1390,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
           <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>05/05/2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1467,12 +1467,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
           <t>05/05/2026</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>04/05/2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1508,9 +1508,9 @@
       <c r="I14" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1540,12 +1540,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
           <t>05/05/2026</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>04/05/2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1617,14 +1617,14 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>05/05/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
           <t>04/05/2026</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>03/05/2026</t>
-        </is>
-      </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -1656,11 +1656,11 @@
         </is>
       </c>
       <c r="I16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>0</v>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1690,12 +1690,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>05/05/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
           <t>04/05/2026</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>03/05/2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1767,14 +1767,14 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>04/05/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
           <t>03/05/2026</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>02/05/2026</t>
-        </is>
-      </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -1806,11 +1806,11 @@
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1840,12 +1840,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>04/05/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
           <t>03/05/2026</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1917,14 +1917,14 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
           <t>02/05/2026</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
-        </is>
-      </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -1956,11 +1956,11 @@
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>0</v>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1990,12 +1990,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
           <t>02/05/2026</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2067,14 +2067,14 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>02/05/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
           <t>01/05/2026</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>30/04/2026</t>
-        </is>
-      </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -2106,7 +2106,7 @@
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
@@ -2140,12 +2140,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>02/05/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
           <t>01/05/2026</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>30/04/2026</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2217,12 +2217,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
           <t>30/04/2026</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>29/04/2026</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2290,12 +2290,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
           <t>30/04/2026</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>29/04/2026</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2367,14 +2367,14 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>30/04/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
           <t>29/04/2026</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>28/04/2026</t>
-        </is>
-      </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -2397,7 +2397,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -2405,10 +2405,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I26" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
@@ -2417,39 +2415,37 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Boa</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t>30/04/2026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
           <t>29/04/2026</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>28/04/2026</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2521,14 +2517,14 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>29/04/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
           <t>28/04/2026</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>27/04/2026</t>
-        </is>
-      </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -2551,7 +2547,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2559,8 +2555,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I28" s="2" t="n">
-        <v>0</v>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
@@ -2569,37 +2567,39 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>29/04/2026</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
           <t>28/04/2026</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>27/04/2026</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2671,12 +2671,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>28/04/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
           <t>27/04/2026</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>26/04/2026</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2744,12 +2744,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t>28/04/2026</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
           <t>27/04/2026</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>26/04/2026</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2821,12 +2821,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t>27/04/2026</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
           <t>26/04/2026</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2862,9 +2862,9 @@
       <c r="I32" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -2894,12 +2894,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
+          <t>27/04/2026</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
           <t>26/04/2026</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2971,14 +2971,14 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
           <t>25/04/2026</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>24/04/2026</t>
-        </is>
-      </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -3010,11 +3010,11 @@
         </is>
       </c>
       <c r="I34" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>0</v>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -3044,12 +3044,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
           <t>25/04/2026</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>24/04/2026</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -3121,14 +3121,14 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
           <t>24/04/2026</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>23/04/2026</t>
-        </is>
-      </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -3154,17 +3154,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -3194,12 +3194,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
           <t>24/04/2026</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>23/04/2026</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3271,14 +3271,14 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
+          <t>24/04/2026</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
           <t>23/04/2026</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>22/04/2026</t>
-        </is>
-      </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -3301,33 +3301,33 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>R$ 78,00</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I38" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>0</v>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>14,3%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L38" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>1,1%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
@@ -3344,12 +3344,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
+          <t>24/04/2026</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
           <t>23/04/2026</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>22/04/2026</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -3421,14 +3421,14 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t>23/04/2026</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
           <t>22/04/2026</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -3451,33 +3451,33 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+          <t>R$ 78,00</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J40" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>7</v>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>14,3%</t>
         </is>
       </c>
       <c r="L40" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>1,1%</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
@@ -3494,12 +3494,12 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
+          <t>23/04/2026</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
           <t>22/04/2026</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -3571,14 +3571,14 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>22/04/2026</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
           <t>21/04/2026</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>20/04/2026</t>
-        </is>
-      </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -3601,33 +3601,33 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>R$ 78,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>▼ 75,0%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I42" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>0</v>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>6,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L42" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>1,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3644,12 +3644,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
+          <t>22/04/2026</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
           <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>20/04/2026</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -3721,14 +3721,14 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
           <t>20/04/2026</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>19/04/2026</t>
-        </is>
-      </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -3751,33 +3751,33 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>R$ 312,00</t>
+          <t>R$ 78,00</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>▼ 20,0%</t>
+          <t>▼ 75,0%</t>
         </is>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>15</v>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>6,7%</t>
         </is>
       </c>
       <c r="L44" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>4,0%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
@@ -3794,12 +3794,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
           <t>20/04/2026</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>19/04/2026</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3871,14 +3871,14 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
           <t>19/04/2026</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>18/04/2026</t>
-        </is>
-      </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -3901,33 +3901,33 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>R$ 390,00</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="inlineStr">
-        <is>
-          <t>▲ 66,7%</t>
+          <t>R$ 312,00</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>▼ 20,0%</t>
         </is>
       </c>
       <c r="I46" s="2" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>▼ 4,6%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>8,1%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L46" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>5,2%</t>
+          <t>4,0%</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
@@ -3944,12 +3944,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
           <t>19/04/2026</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -4021,14 +4021,14 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
           <t>18/04/2026</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>17/04/2026</t>
-        </is>
-      </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -4051,33 +4051,33 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>R$ 234,00</t>
-        </is>
-      </c>
-      <c r="H48" s="3" t="inlineStr">
-        <is>
-          <t>▼ 49,9%</t>
+          <t>R$ 390,00</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>▲ 66,7%</t>
         </is>
       </c>
       <c r="I48" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>▼ 28,6%</t>
+          <t>▼ 4,6%</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>4,6%</t>
+          <t>8,1%</t>
         </is>
       </c>
       <c r="L48" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>3,6%</t>
+          <t>5,2%</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
@@ -4094,12 +4094,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
           <t>18/04/2026</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>17/04/2026</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -4171,14 +4171,14 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
           <t>17/04/2026</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>16/04/2026</t>
-        </is>
-      </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -4201,33 +4201,33 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>R$ 467,00</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="inlineStr">
-        <is>
-          <t>▲ 199,4%</t>
+          <t>R$ 234,00</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>▼ 49,9%</t>
         </is>
       </c>
       <c r="I50" s="2" t="n">
-        <v>91</v>
-      </c>
-      <c r="J50" s="4" t="inlineStr">
-        <is>
-          <t>▲ 49,2%</t>
+        <v>65</v>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>▼ 28,6%</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>6,6%</t>
+          <t>4,6%</t>
         </is>
       </c>
       <c r="L50" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>4,7%</t>
+          <t>3,6%</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
@@ -4244,12 +4244,12 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
           <t>17/04/2026</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>16/04/2026</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -4321,14 +4321,14 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
+          <t>17/04/2026</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
           <t>16/04/2026</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>15/04/2026</t>
-        </is>
-      </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -4351,33 +4351,33 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>R$ 156,00</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="inlineStr">
-        <is>
-          <t>▼ 33,3%</t>
+          <t>R$ 467,00</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>▲ 199,4%</t>
         </is>
       </c>
       <c r="I52" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="J52" s="3" t="inlineStr">
-        <is>
-          <t>▼ 19,7%</t>
+        <v>91</v>
+      </c>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>▲ 49,2%</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>3,3%</t>
+          <t>6,6%</t>
         </is>
       </c>
       <c r="L52" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>1,7%</t>
+          <t>4,7%</t>
         </is>
       </c>
       <c r="N52" s="2" t="inlineStr">
@@ -4394,12 +4394,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
+          <t>17/04/2026</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
           <t>16/04/2026</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>15/04/2026</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -4471,14 +4471,14 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
+          <t>16/04/2026</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
           <t>15/04/2026</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>14/04/2026</t>
-        </is>
-      </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -4501,33 +4501,33 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>R$ 234,00</t>
+          <t>R$ 156,00</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>▼ 49,9%</t>
+          <t>▼ 33,3%</t>
         </is>
       </c>
       <c r="I54" s="2" t="n">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>▼ 2,6%</t>
+          <t>▼ 19,7%</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>3,9%</t>
+          <t>3,3%</t>
         </is>
       </c>
       <c r="L54" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>2,1%</t>
+          <t>1,7%</t>
         </is>
       </c>
       <c r="N54" s="2" t="inlineStr">
@@ -4544,12 +4544,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
+          <t>16/04/2026</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
           <t>15/04/2026</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>14/04/2026</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -4621,14 +4621,14 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
+          <t>15/04/2026</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
           <t>14/04/2026</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>13/04/2026</t>
-        </is>
-      </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -4651,33 +4651,33 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>R$ 467,00</t>
+          <t>R$ 234,00</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>▼ 14,3%</t>
+          <t>▼ 49,9%</t>
         </is>
       </c>
       <c r="I56" s="2" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>▼ 27,1%</t>
+          <t>▼ 2,6%</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>7,7%</t>
+          <t>3,9%</t>
         </is>
       </c>
       <c r="L56" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>4,3%</t>
+          <t>2,1%</t>
         </is>
       </c>
       <c r="N56" s="2" t="inlineStr">
@@ -4694,12 +4694,12 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
+          <t>15/04/2026</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
           <t>14/04/2026</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>13/04/2026</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -4771,14 +4771,14 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
+          <t>14/04/2026</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
           <t>13/04/2026</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -4801,33 +4801,33 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>R$ 545,00</t>
-        </is>
-      </c>
-      <c r="H58" s="4" t="inlineStr">
-        <is>
-          <t>▲ 74,7%</t>
+          <t>R$ 467,00</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>▼ 14,3%</t>
         </is>
       </c>
       <c r="I58" s="2" t="n">
-        <v>107</v>
-      </c>
-      <c r="J58" s="4" t="inlineStr">
-        <is>
-          <t>▲ 10,3%</t>
+        <v>78</v>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>▼ 27,1%</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>6,5%</t>
+          <t>7,7%</t>
         </is>
       </c>
       <c r="L58" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>4,5%</t>
+          <t>4,3%</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr">
@@ -4844,14 +4844,14 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
+          <t>14/04/2026</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
           <t>13/04/2026</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -4882,8 +4882,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I59" s="2" t="n">
-        <v>0</v>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
@@ -4892,39 +4894,41 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L59" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
+          <t>13/04/2026</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
           <t>12/04/2026</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>11/04/2026</t>
-        </is>
-      </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -4947,33 +4951,33 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>R$ 312,00</t>
+          <t>R$ 545,00</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr">
         <is>
-          <t>▲ 300,0%</t>
+          <t>▲ 74,7%</t>
         </is>
       </c>
       <c r="I60" s="2" t="n">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="J60" s="4" t="inlineStr">
         <is>
-          <t>▲ 203,1%</t>
+          <t>▲ 10,3%</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>4,1%</t>
+          <t>6,5%</t>
         </is>
       </c>
       <c r="L60" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>4,7%</t>
+          <t>4,5%</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
@@ -4990,12 +4994,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
+          <t>13/04/2026</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
           <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>11/04/2026</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -5063,14 +5067,14 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
           <t>11/04/2026</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>10/04/2026</t>
-        </is>
-      </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -5093,38 +5097,38 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>R$ 78,00</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 312,00</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>▲ 300,0%</t>
         </is>
       </c>
       <c r="I62" s="2" t="n">
-        <v>32</v>
+        <v>97</v>
       </c>
       <c r="J62" s="4" t="inlineStr">
         <is>
-          <t>▲ 1500,0%</t>
+          <t>▲ 203,1%</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>3,1%</t>
+          <t>4,1%</t>
         </is>
       </c>
       <c r="L62" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>1,0%</t>
+          <t>4,7%</t>
         </is>
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O62" s="2" t="inlineStr">
@@ -5136,12 +5140,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
           <t>11/04/2026</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>10/04/2026</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -5177,9 +5181,9 @@
       <c r="I63" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J63" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -5209,14 +5213,14 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
           <t>10/04/2026</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>09/04/2026</t>
-        </is>
-      </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -5239,7 +5243,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 78,00</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -5248,29 +5252,29 @@
         </is>
       </c>
       <c r="I64" s="2" t="n">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="J64" s="4" t="inlineStr">
         <is>
-          <t>▲ 100,0%</t>
+          <t>▲ 1500,0%</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>3,1%</t>
         </is>
       </c>
       <c r="L64" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Sem calcular</t>
         </is>
       </c>
       <c r="O64" s="2" t="inlineStr">
@@ -5282,14 +5286,14 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
           <t>10/04/2026</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>09/04/2026</t>
-        </is>
-      </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -5315,17 +5319,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H65" s="3" t="inlineStr">
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
         <is>
           <t>▼ 100,0%</t>
-        </is>
-      </c>
-      <c r="I65" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="J65" s="4" t="inlineStr">
-        <is>
-          <t>▲ 200,0%</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
@@ -5355,14 +5359,14 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
+          <t>10/04/2026</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
           <t>09/04/2026</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>08/04/2026</t>
-        </is>
-      </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -5388,17 +5392,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H66" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I66" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J66" s="3" t="inlineStr">
-        <is>
-          <t>▼ 99,2%</t>
+        <v>2</v>
+      </c>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
@@ -5428,14 +5432,14 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
+          <t>10/04/2026</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
           <t>09/04/2026</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>08/04/2026</t>
-        </is>
-      </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -5458,33 +5462,33 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>R$ 75,00</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I67" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J67" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>6</v>
+      </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>▲ 200,0%</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>50,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L67" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>1,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N67" s="2" t="inlineStr">
@@ -5501,14 +5505,14 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
           <t>08/04/2026</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>07/04/2026</t>
-        </is>
-      </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -5531,33 +5535,33 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>R$ 659,00</t>
-        </is>
-      </c>
-      <c r="H68" s="4" t="inlineStr">
-        <is>
-          <t>▲ 124,9%</t>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I68" s="2" t="n">
-        <v>120</v>
-      </c>
-      <c r="J68" s="4" t="inlineStr">
-        <is>
-          <t>▲ 4,3%</t>
+        <v>1</v>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>▼ 99,2%</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>7,5%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L68" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>6,5%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N68" s="2" t="inlineStr">
@@ -5574,14 +5578,14 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
           <t>08/04/2026</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>07/04/2026</t>
-        </is>
-      </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -5604,33 +5608,33 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
-        </is>
-      </c>
-      <c r="H69" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+          <t>R$ 75,00</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J69" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>2</v>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>50,0%</t>
         </is>
       </c>
       <c r="L69" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M69" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N69" s="2" t="inlineStr">
@@ -5647,14 +5651,14 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
+          <t>08/04/2026</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
           <t>07/04/2026</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>06/04/2026</t>
-        </is>
-      </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -5677,38 +5681,38 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>R$ 293,00</t>
-        </is>
-      </c>
-      <c r="H70" s="3" t="inlineStr">
-        <is>
-          <t>▼ 33,3%</t>
+          <t>R$ 659,00</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>▲ 124,9%</t>
         </is>
       </c>
       <c r="I70" s="2" t="n">
-        <v>115</v>
-      </c>
-      <c r="J70" s="3" t="inlineStr">
-        <is>
-          <t>▼ 12,2%</t>
+        <v>120</v>
+      </c>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>▲ 4,3%</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>3,5%</t>
+          <t>7,5%</t>
         </is>
       </c>
       <c r="L70" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="M70" s="2" t="inlineStr">
         <is>
-          <t>2,8%</t>
+          <t>6,5%</t>
         </is>
       </c>
       <c r="N70" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O70" s="2" t="inlineStr">
@@ -5720,14 +5724,14 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
+          <t>08/04/2026</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
           <t>07/04/2026</t>
         </is>
       </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>06/04/2026</t>
-        </is>
-      </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -5750,33 +5754,33 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>R$ 75,00</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I71" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>▼ 12,5%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>14,3%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L71" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>0,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N71" s="2" t="inlineStr">
@@ -5793,14 +5797,14 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
           <t>06/04/2026</t>
         </is>
       </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>05/04/2026</t>
-        </is>
-      </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -5823,38 +5827,38 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>R$ 439,00</t>
+          <t>R$ 293,00</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>▼ 25,1%</t>
+          <t>▼ 33,3%</t>
         </is>
       </c>
       <c r="I72" s="2" t="n">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>▼ 0,8%</t>
+          <t>▼ 12,2%</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>4,6%</t>
+          <t>3,5%</t>
         </is>
       </c>
       <c r="L72" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>4,8%</t>
+          <t>2,8%</t>
         </is>
       </c>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Sem calcular</t>
         </is>
       </c>
       <c r="O72" s="2" t="inlineStr">
@@ -5866,14 +5870,14 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
           <t>06/04/2026</t>
         </is>
       </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>05/04/2026</t>
-        </is>
-      </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -5896,7 +5900,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 75,00</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -5905,24 +5909,24 @@
         </is>
       </c>
       <c r="I73" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>▼ 20,0%</t>
+          <t>▼ 12,5%</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>14,3%</t>
         </is>
       </c>
       <c r="L73" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,7%</t>
         </is>
       </c>
       <c r="N73" s="2" t="inlineStr">
@@ -5939,14 +5943,14 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
+          <t>06/04/2026</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
           <t>05/04/2026</t>
         </is>
       </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>04/04/2026</t>
-        </is>
-      </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -5969,33 +5973,33 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>R$ 586,00</t>
+          <t>R$ 439,00</t>
         </is>
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>▼ 11,1%</t>
+          <t>▼ 25,1%</t>
         </is>
       </c>
       <c r="I74" s="2" t="n">
-        <v>132</v>
-      </c>
-      <c r="J74" s="4" t="inlineStr">
-        <is>
-          <t>▲ 34,7%</t>
+        <v>131</v>
+      </c>
+      <c r="J74" s="3" t="inlineStr">
+        <is>
+          <t>▼ 0,8%</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>6,1%</t>
+          <t>4,6%</t>
         </is>
       </c>
       <c r="L74" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>6,8%</t>
+          <t>4,8%</t>
         </is>
       </c>
       <c r="N74" s="2" t="inlineStr">
@@ -6012,14 +6016,14 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
+          <t>06/04/2026</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
           <t>05/04/2026</t>
         </is>
       </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>04/04/2026</t>
-        </is>
-      </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -6045,17 +6049,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H75" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I75" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J75" s="4" t="inlineStr">
-        <is>
-          <t>▲ 25,0%</t>
+        <v>8</v>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>▼ 20,0%</t>
         </is>
       </c>
       <c r="K75" s="2" t="inlineStr">
@@ -6085,14 +6089,14 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
           <t>04/04/2026</t>
         </is>
       </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>03/04/2026</t>
-        </is>
-      </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -6115,33 +6119,33 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>R$ 659,00</t>
-        </is>
-      </c>
-      <c r="H76" s="4" t="inlineStr">
-        <is>
-          <t>▲ 80,1%</t>
+          <t>R$ 586,00</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>▼ 11,1%</t>
         </is>
       </c>
       <c r="I76" s="2" t="n">
-        <v>98</v>
+        <v>132</v>
       </c>
       <c r="J76" s="4" t="inlineStr">
         <is>
-          <t>▲ 3,2%</t>
+          <t>▲ 34,7%</t>
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>9,2%</t>
+          <t>6,1%</t>
         </is>
       </c>
       <c r="L76" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>6,3%</t>
+          <t>6,8%</t>
         </is>
       </c>
       <c r="N76" s="2" t="inlineStr">
@@ -6158,14 +6162,14 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
           <t>04/04/2026</t>
         </is>
       </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>03/04/2026</t>
-        </is>
-      </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -6188,33 +6192,33 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>R$ 75,00</t>
-        </is>
-      </c>
-      <c r="H77" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I77" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J77" s="4" t="inlineStr">
         <is>
-          <t>▲ 14,3%</t>
+          <t>▲ 25,0%</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>12,5%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L77" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M77" s="2" t="inlineStr">
         <is>
-          <t>0,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N77" s="2" t="inlineStr">
@@ -6231,14 +6235,14 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
+          <t>04/04/2026</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
           <t>03/04/2026</t>
         </is>
       </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>02/04/2026</t>
-        </is>
-      </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -6261,33 +6265,33 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>R$ 366,00</t>
-        </is>
-      </c>
-      <c r="H78" s="3" t="inlineStr">
-        <is>
-          <t>▼ 61,6%</t>
+          <t>R$ 659,00</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>▲ 80,1%</t>
         </is>
       </c>
       <c r="I78" s="2" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J78" s="4" t="inlineStr">
         <is>
-          <t>▲ 13,1%</t>
+          <t>▲ 3,2%</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>5,3%</t>
+          <t>9,2%</t>
         </is>
       </c>
       <c r="L78" s="2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="M78" s="2" t="inlineStr">
         <is>
-          <t>4,8%</t>
+          <t>6,3%</t>
         </is>
       </c>
       <c r="N78" s="2" t="inlineStr">
@@ -6304,14 +6308,14 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
+          <t>04/04/2026</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
           <t>03/04/2026</t>
         </is>
       </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>02/04/2026</t>
-        </is>
-      </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -6334,7 +6338,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 75,00</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -6343,24 +6347,24 @@
         </is>
       </c>
       <c r="I79" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="J79" s="3" t="inlineStr">
-        <is>
-          <t>▼ 63,2%</t>
+        <v>8</v>
+      </c>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>▲ 14,3%</t>
         </is>
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>12,5%</t>
         </is>
       </c>
       <c r="L79" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M79" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,7%</t>
         </is>
       </c>
       <c r="N79" s="2" t="inlineStr">
@@ -6377,14 +6381,14 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
           <t>02/04/2026</t>
         </is>
       </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>01/04/2026</t>
-        </is>
-      </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -6407,33 +6411,33 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>R$ 952,00</t>
-        </is>
-      </c>
-      <c r="H80" s="4" t="inlineStr">
-        <is>
-          <t>▲ 210,1%</t>
+          <t>R$ 366,00</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>▼ 61,6%</t>
         </is>
       </c>
       <c r="I80" s="2" t="n">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="J80" s="4" t="inlineStr">
         <is>
-          <t>▲ 1,2%</t>
+          <t>▲ 13,1%</t>
         </is>
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>15,5%</t>
+          <t>5,3%</t>
         </is>
       </c>
       <c r="L80" s="2" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="M80" s="2" t="inlineStr">
         <is>
-          <t>11,3%</t>
+          <t>4,8%</t>
         </is>
       </c>
       <c r="N80" s="2" t="inlineStr">
@@ -6450,14 +6454,14 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
           <t>02/04/2026</t>
         </is>
       </c>
-      <c r="B81" s="2" t="inlineStr">
-        <is>
-          <t>01/04/2026</t>
-        </is>
-      </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -6489,11 +6493,11 @@
         </is>
       </c>
       <c r="I81" s="2" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>▼ 26,9%</t>
+          <t>▼ 63,2%</t>
         </is>
       </c>
       <c r="K81" s="2" t="inlineStr">
@@ -6523,14 +6527,14 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
           <t>01/04/2026</t>
         </is>
       </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>31/03/2026</t>
-        </is>
-      </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -6553,33 +6557,33 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>R$ 307,00</t>
-        </is>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 952,00</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>▲ 210,1%</t>
         </is>
       </c>
       <c r="I82" s="2" t="n">
-        <v>83</v>
-      </c>
-      <c r="J82" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>84</v>
+      </c>
+      <c r="J82" s="4" t="inlineStr">
+        <is>
+          <t>▲ 1,2%</t>
         </is>
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>4,8%</t>
+          <t>15,5%</t>
         </is>
       </c>
       <c r="L82" s="2" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="M82" s="2" t="inlineStr">
         <is>
-          <t>3,3%</t>
+          <t>11,3%</t>
         </is>
       </c>
       <c r="N82" s="2" t="inlineStr">
@@ -6596,14 +6600,14 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
           <t>01/04/2026</t>
         </is>
       </c>
-      <c r="B83" s="2" t="inlineStr">
-        <is>
-          <t>31/03/2026</t>
-        </is>
-      </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
           <t>BRINQ-019</t>
@@ -6635,11 +6639,11 @@
         </is>
       </c>
       <c r="I83" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="J83" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>19</v>
+      </c>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>▼ 26,9%</t>
         </is>
       </c>
       <c r="K83" s="2" t="inlineStr">
@@ -6666,8 +6670,154 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>31/03/2026</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>3076915307</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>R$ 77,90</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>R$ 307,00</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>4,8%</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>3,3%</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>31/03/2026</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>6311164080</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>R$ 78,80</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O85" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O83"/>
+  <autoFilter ref="A1:O85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
relatorios 14-05 e 15-05
</commit_message>
<xml_diff>
--- a/saida_skus/SKU_BRINQ-019-VASSOURA-INFANTIL-UNICORNIO.xlsx
+++ b/saida_skus/SKU_BRINQ-019-VASSOURA-INFANTIL-UNICORNIO.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Analise" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analise'!$A$1:$O$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analise'!$A$1:$O$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O85"/>
+  <dimension ref="A1:O91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -559,12 +559,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>12/05/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>14/05/2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -632,12 +632,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>12/05/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>14/05/2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -709,12 +709,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>14/05/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>10/05/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -747,8 +747,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n">
-        <v>0</v>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -757,37 +759,39 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>14/05/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>10/05/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -859,12 +863,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>10/05/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>12/05/2026</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -889,7 +893,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -897,10 +901,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I6" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -909,39 +911,37 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Boa</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>10/05/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>12/05/2026</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1013,12 +1013,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>12/05/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1051,10 +1051,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I8" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -1063,39 +1061,37 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Boa</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>12/05/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1167,12 +1163,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1240,12 +1236,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1317,12 +1313,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1347,7 +1343,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1355,8 +1351,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I12" s="2" t="n">
-        <v>0</v>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
@@ -1365,37 +1363,39 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1467,12 +1467,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1505,8 +1505,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I14" s="2" t="n">
-        <v>0</v>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
@@ -1515,37 +1517,39 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1617,12 +1621,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1658,9 +1662,9 @@
       <c r="I16" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1690,12 +1694,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1767,12 +1771,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1806,7 +1810,7 @@
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
@@ -1840,12 +1844,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1917,12 +1921,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1958,9 +1962,9 @@
       <c r="I20" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1990,12 +1994,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2067,12 +2071,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2106,11 +2110,11 @@
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>0</v>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -2140,12 +2144,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2217,12 +2221,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2256,7 +2260,7 @@
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
@@ -2290,12 +2294,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2367,12 +2371,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2408,9 +2412,9 @@
       <c r="I26" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2440,12 +2444,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2517,12 +2521,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2547,7 +2551,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2555,10 +2559,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I28" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
@@ -2567,39 +2569,37 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Boa</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2671,12 +2671,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2744,12 +2744,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2821,12 +2821,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2894,12 +2894,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2971,12 +2971,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -3009,47 +3009,51 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -3121,12 +3125,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3160,7 +3164,7 @@
         </is>
       </c>
       <c r="I36" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
@@ -3194,12 +3198,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3271,12 +3275,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -3304,17 +3308,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H38" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I38" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J38" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -3344,12 +3348,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -3421,12 +3425,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -3451,7 +3455,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>R$ 78,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -3460,24 +3464,24 @@
         </is>
       </c>
       <c r="I40" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>0</v>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>14,3%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L40" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>1,1%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
@@ -3494,12 +3498,12 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -3571,12 +3575,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -3604,17 +3608,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I42" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -3644,12 +3648,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -3721,12 +3725,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -3751,33 +3755,33 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>R$ 78,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>▼ 75,0%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I44" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>0</v>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>6,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L44" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>1,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
@@ -3794,12 +3798,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3871,12 +3875,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3901,33 +3905,33 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>R$ 312,00</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="inlineStr">
-        <is>
-          <t>▼ 20,0%</t>
+          <t>R$ 78,00</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I46" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J46" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>7</v>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>14,3%</t>
         </is>
       </c>
       <c r="L46" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>4,0%</t>
+          <t>1,1%</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
@@ -3944,12 +3948,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -4021,12 +4025,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -4051,33 +4055,33 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>R$ 390,00</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>▲ 66,7%</t>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I48" s="2" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>▼ 4,6%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>8,1%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L48" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>5,2%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
@@ -4094,12 +4098,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -4171,12 +4175,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -4201,33 +4205,33 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>R$ 234,00</t>
+          <t>R$ 78,00</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>▼ 49,9%</t>
+          <t>▼ 75,0%</t>
         </is>
       </c>
       <c r="I50" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="J50" s="3" t="inlineStr">
-        <is>
-          <t>▼ 28,6%</t>
+        <v>15</v>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>4,6%</t>
+          <t>6,7%</t>
         </is>
       </c>
       <c r="L50" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>3,6%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
@@ -4244,12 +4248,12 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -4321,12 +4325,12 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -4351,33 +4355,33 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>R$ 467,00</t>
-        </is>
-      </c>
-      <c r="H52" s="4" t="inlineStr">
-        <is>
-          <t>▲ 199,4%</t>
+          <t>R$ 312,00</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>▼ 20,0%</t>
         </is>
       </c>
       <c r="I52" s="2" t="n">
-        <v>91</v>
-      </c>
-      <c r="J52" s="4" t="inlineStr">
-        <is>
-          <t>▲ 49,2%</t>
+        <v>0</v>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>6,6%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L52" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>4,7%</t>
+          <t>4,0%</t>
         </is>
       </c>
       <c r="N52" s="2" t="inlineStr">
@@ -4394,12 +4398,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -4471,12 +4475,12 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -4501,33 +4505,33 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>R$ 156,00</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr">
-        <is>
-          <t>▼ 33,3%</t>
+          <t>R$ 390,00</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>▲ 66,7%</t>
         </is>
       </c>
       <c r="I54" s="2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>▼ 19,7%</t>
+          <t>▼ 4,6%</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>3,3%</t>
+          <t>8,1%</t>
         </is>
       </c>
       <c r="L54" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>1,7%</t>
+          <t>5,2%</t>
         </is>
       </c>
       <c r="N54" s="2" t="inlineStr">
@@ -4544,12 +4548,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -4621,12 +4625,12 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -4660,16 +4664,16 @@
         </is>
       </c>
       <c r="I56" s="2" t="n">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>▼ 2,6%</t>
+          <t>▼ 28,6%</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>3,9%</t>
+          <t>4,6%</t>
         </is>
       </c>
       <c r="L56" s="2" t="n">
@@ -4677,7 +4681,7 @@
       </c>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>2,1%</t>
+          <t>3,6%</t>
         </is>
       </c>
       <c r="N56" s="2" t="inlineStr">
@@ -4694,12 +4698,12 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -4771,12 +4775,12 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -4804,22 +4808,22 @@
           <t>R$ 467,00</t>
         </is>
       </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>▼ 14,3%</t>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>▲ 199,4%</t>
         </is>
       </c>
       <c r="I58" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="J58" s="3" t="inlineStr">
-        <is>
-          <t>▼ 27,1%</t>
+        <v>91</v>
+      </c>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>▲ 49,2%</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>7,7%</t>
+          <t>6,6%</t>
         </is>
       </c>
       <c r="L58" s="2" t="n">
@@ -4827,7 +4831,7 @@
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>4,3%</t>
+          <t>4,7%</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr">
@@ -4844,12 +4848,12 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -4921,12 +4925,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -4951,33 +4955,33 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>R$ 545,00</t>
-        </is>
-      </c>
-      <c r="H60" s="4" t="inlineStr">
-        <is>
-          <t>▲ 74,7%</t>
+          <t>R$ 156,00</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>▼ 33,3%</t>
         </is>
       </c>
       <c r="I60" s="2" t="n">
-        <v>107</v>
-      </c>
-      <c r="J60" s="4" t="inlineStr">
-        <is>
-          <t>▲ 10,3%</t>
+        <v>61</v>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>▼ 19,7%</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>6,5%</t>
+          <t>3,3%</t>
         </is>
       </c>
       <c r="L60" s="2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>4,5%</t>
+          <t>1,7%</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
@@ -4994,12 +4998,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -5024,7 +5028,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -5032,8 +5036,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I61" s="2" t="n">
-        <v>0</v>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
@@ -5042,37 +5048,39 @@
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L61" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M61" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N61" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -5097,33 +5105,33 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>R$ 312,00</t>
-        </is>
-      </c>
-      <c r="H62" s="4" t="inlineStr">
-        <is>
-          <t>▲ 300,0%</t>
+          <t>R$ 234,00</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>▼ 49,9%</t>
         </is>
       </c>
       <c r="I62" s="2" t="n">
-        <v>97</v>
-      </c>
-      <c r="J62" s="4" t="inlineStr">
-        <is>
-          <t>▲ 203,1%</t>
+        <v>76</v>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>▼ 2,6%</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>4,1%</t>
+          <t>3,9%</t>
         </is>
       </c>
       <c r="L62" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>4,7%</t>
+          <t>2,1%</t>
         </is>
       </c>
       <c r="N62" s="2" t="inlineStr">
@@ -5140,12 +5148,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -5170,7 +5178,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -5178,8 +5186,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I63" s="2" t="n">
-        <v>0</v>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
@@ -5188,37 +5198,39 @@
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L63" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N63" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -5243,38 +5255,38 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>R$ 78,00</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 467,00</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>▼ 14,3%</t>
         </is>
       </c>
       <c r="I64" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="J64" s="4" t="inlineStr">
-        <is>
-          <t>▲ 1500,0%</t>
+        <v>78</v>
+      </c>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>▼ 27,1%</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>3,1%</t>
+          <t>7,7%</t>
         </is>
       </c>
       <c r="L64" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>1,0%</t>
+          <t>4,3%</t>
         </is>
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O64" s="2" t="inlineStr">
@@ -5286,12 +5298,12 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -5316,7 +5328,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -5324,47 +5336,51 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L65" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -5389,33 +5405,33 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 545,00</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>▲ 74,7%</t>
         </is>
       </c>
       <c r="I66" s="2" t="n">
-        <v>2</v>
+        <v>107</v>
       </c>
       <c r="J66" s="4" t="inlineStr">
         <is>
-          <t>▲ 100,0%</t>
+          <t>▲ 10,3%</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>6,5%</t>
         </is>
       </c>
       <c r="L66" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>4,5%</t>
         </is>
       </c>
       <c r="N66" s="2" t="inlineStr">
@@ -5432,12 +5448,12 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -5465,17 +5481,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H67" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I67" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="J67" s="4" t="inlineStr">
-        <is>
-          <t>▲ 200,0%</t>
+        <v>0</v>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr">
@@ -5505,12 +5521,12 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -5535,33 +5551,33 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
-        </is>
-      </c>
-      <c r="H68" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+          <t>R$ 312,00</t>
+        </is>
+      </c>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>▲ 300,0%</t>
         </is>
       </c>
       <c r="I68" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J68" s="3" t="inlineStr">
-        <is>
-          <t>▼ 99,2%</t>
+        <v>97</v>
+      </c>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t>▲ 203,1%</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>4,1%</t>
         </is>
       </c>
       <c r="L68" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>4,7%</t>
         </is>
       </c>
       <c r="N68" s="2" t="inlineStr">
@@ -5578,12 +5594,12 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -5608,7 +5624,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>R$ 75,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -5617,7 +5633,7 @@
         </is>
       </c>
       <c r="I69" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
@@ -5626,15 +5642,15 @@
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>50,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L69" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M69" s="2" t="inlineStr">
         <is>
-          <t>1,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N69" s="2" t="inlineStr">
@@ -5651,12 +5667,12 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -5681,38 +5697,38 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>R$ 659,00</t>
-        </is>
-      </c>
-      <c r="H70" s="4" t="inlineStr">
-        <is>
-          <t>▲ 124,9%</t>
+          <t>R$ 78,00</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I70" s="2" t="n">
-        <v>120</v>
+        <v>32</v>
       </c>
       <c r="J70" s="4" t="inlineStr">
         <is>
-          <t>▲ 4,3%</t>
+          <t>▲ 1500,0%</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>7,5%</t>
+          <t>3,1%</t>
         </is>
       </c>
       <c r="L70" s="2" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="M70" s="2" t="inlineStr">
         <is>
-          <t>6,5%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N70" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Sem calcular</t>
         </is>
       </c>
       <c r="O70" s="2" t="inlineStr">
@@ -5724,12 +5740,12 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -5757,9 +5773,9 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H71" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I71" s="2" t="n">
@@ -5797,12 +5813,12 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -5827,38 +5843,38 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>R$ 293,00</t>
-        </is>
-      </c>
-      <c r="H72" s="3" t="inlineStr">
-        <is>
-          <t>▼ 33,3%</t>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I72" s="2" t="n">
-        <v>115</v>
-      </c>
-      <c r="J72" s="3" t="inlineStr">
-        <is>
-          <t>▼ 12,2%</t>
+        <v>2</v>
+      </c>
+      <c r="J72" s="4" t="inlineStr">
+        <is>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>3,5%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L72" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>2,8%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O72" s="2" t="inlineStr">
@@ -5870,12 +5886,12 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -5900,33 +5916,33 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>R$ 75,00</t>
-        </is>
-      </c>
-      <c r="H73" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I73" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="J73" s="3" t="inlineStr">
-        <is>
-          <t>▼ 12,5%</t>
+        <v>6</v>
+      </c>
+      <c r="J73" s="4" t="inlineStr">
+        <is>
+          <t>▲ 200,0%</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>14,3%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L73" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>0,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N73" s="2" t="inlineStr">
@@ -5943,12 +5959,12 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -5973,33 +5989,33 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>R$ 439,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>▼ 25,1%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I74" s="2" t="n">
-        <v>131</v>
+        <v>1</v>
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>▼ 0,8%</t>
+          <t>▼ 99,2%</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>4,6%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L74" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>4,8%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N74" s="2" t="inlineStr">
@@ -6016,12 +6032,12 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -6046,7 +6062,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 75,00</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -6055,24 +6071,24 @@
         </is>
       </c>
       <c r="I75" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="J75" s="3" t="inlineStr">
-        <is>
-          <t>▼ 20,0%</t>
+        <v>2</v>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>50,0%</t>
         </is>
       </c>
       <c r="L75" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N75" s="2" t="inlineStr">
@@ -6089,12 +6105,12 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -6119,33 +6135,33 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>R$ 586,00</t>
-        </is>
-      </c>
-      <c r="H76" s="3" t="inlineStr">
-        <is>
-          <t>▼ 11,1%</t>
+          <t>R$ 659,00</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>▲ 124,9%</t>
         </is>
       </c>
       <c r="I76" s="2" t="n">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J76" s="4" t="inlineStr">
         <is>
-          <t>▲ 34,7%</t>
+          <t>▲ 4,3%</t>
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>6,1%</t>
+          <t>7,5%</t>
         </is>
       </c>
       <c r="L76" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>6,8%</t>
+          <t>6,5%</t>
         </is>
       </c>
       <c r="N76" s="2" t="inlineStr">
@@ -6162,12 +6178,12 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -6201,11 +6217,11 @@
         </is>
       </c>
       <c r="I77" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J77" s="4" t="inlineStr">
-        <is>
-          <t>▲ 25,0%</t>
+        <v>0</v>
+      </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr">
@@ -6235,12 +6251,12 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -6265,38 +6281,38 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>R$ 659,00</t>
-        </is>
-      </c>
-      <c r="H78" s="4" t="inlineStr">
-        <is>
-          <t>▲ 80,1%</t>
+          <t>R$ 293,00</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>▼ 33,3%</t>
         </is>
       </c>
       <c r="I78" s="2" t="n">
-        <v>98</v>
-      </c>
-      <c r="J78" s="4" t="inlineStr">
-        <is>
-          <t>▲ 3,2%</t>
+        <v>115</v>
+      </c>
+      <c r="J78" s="3" t="inlineStr">
+        <is>
+          <t>▼ 12,2%</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>9,2%</t>
+          <t>3,5%</t>
         </is>
       </c>
       <c r="L78" s="2" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="M78" s="2" t="inlineStr">
         <is>
-          <t>6,3%</t>
+          <t>2,8%</t>
         </is>
       </c>
       <c r="N78" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Sem calcular</t>
         </is>
       </c>
       <c r="O78" s="2" t="inlineStr">
@@ -6308,12 +6324,12 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -6347,16 +6363,16 @@
         </is>
       </c>
       <c r="I79" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="J79" s="4" t="inlineStr">
-        <is>
-          <t>▲ 14,3%</t>
+        <v>7</v>
+      </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>▼ 12,5%</t>
         </is>
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>12,5%</t>
+          <t>14,3%</t>
         </is>
       </c>
       <c r="L79" s="2" t="n">
@@ -6381,12 +6397,12 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -6411,29 +6427,29 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>R$ 366,00</t>
+          <t>R$ 439,00</t>
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>▼ 61,6%</t>
+          <t>▼ 25,1%</t>
         </is>
       </c>
       <c r="I80" s="2" t="n">
-        <v>95</v>
-      </c>
-      <c r="J80" s="4" t="inlineStr">
-        <is>
-          <t>▲ 13,1%</t>
+        <v>131</v>
+      </c>
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t>▼ 0,8%</t>
         </is>
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>5,3%</t>
+          <t>4,6%</t>
         </is>
       </c>
       <c r="L80" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M80" s="2" t="inlineStr">
         <is>
@@ -6454,12 +6470,12 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -6493,11 +6509,11 @@
         </is>
       </c>
       <c r="I81" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>▼ 63,2%</t>
+          <t>▼ 20,0%</t>
         </is>
       </c>
       <c r="K81" s="2" t="inlineStr">
@@ -6527,12 +6543,12 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -6557,33 +6573,33 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>R$ 952,00</t>
-        </is>
-      </c>
-      <c r="H82" s="4" t="inlineStr">
-        <is>
-          <t>▲ 210,1%</t>
+          <t>R$ 586,00</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>▼ 11,1%</t>
         </is>
       </c>
       <c r="I82" s="2" t="n">
-        <v>84</v>
+        <v>132</v>
       </c>
       <c r="J82" s="4" t="inlineStr">
         <is>
-          <t>▲ 1,2%</t>
+          <t>▲ 34,7%</t>
         </is>
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>15,5%</t>
+          <t>6,1%</t>
         </is>
       </c>
       <c r="L82" s="2" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="M82" s="2" t="inlineStr">
         <is>
-          <t>11,3%</t>
+          <t>6,8%</t>
         </is>
       </c>
       <c r="N82" s="2" t="inlineStr">
@@ -6600,12 +6616,12 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -6633,17 +6649,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H83" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I83" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="J83" s="3" t="inlineStr">
-        <is>
-          <t>▼ 26,9%</t>
+        <v>10</v>
+      </c>
+      <c r="J83" s="4" t="inlineStr">
+        <is>
+          <t>▲ 25,0%</t>
         </is>
       </c>
       <c r="K83" s="2" t="inlineStr">
@@ -6673,12 +6689,12 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>03/04/2026</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -6703,33 +6719,33 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>R$ 307,00</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 659,00</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>▲ 80,1%</t>
         </is>
       </c>
       <c r="I84" s="2" t="n">
-        <v>83</v>
-      </c>
-      <c r="J84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>98</v>
+      </c>
+      <c r="J84" s="4" t="inlineStr">
+        <is>
+          <t>▲ 3,2%</t>
         </is>
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t>4,8%</t>
+          <t>9,2%</t>
         </is>
       </c>
       <c r="L84" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="M84" s="2" t="inlineStr">
         <is>
-          <t>3,3%</t>
+          <t>6,3%</t>
         </is>
       </c>
       <c r="N84" s="2" t="inlineStr">
@@ -6746,78 +6762,516 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
+          <t>04/04/2026</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>6311164080</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>R$ 78,80</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>R$ 75,00</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J85" s="4" t="inlineStr">
+        <is>
+          <t>▲ 14,3%</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>12,5%</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>0,7%</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O85" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>3076915307</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>R$ 77,90</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>R$ 366,00</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>▼ 61,6%</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="J86" s="4" t="inlineStr">
+        <is>
+          <t>▲ 13,1%</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>5,3%</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>4,8%</t>
+        </is>
+      </c>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>6311164080</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>R$ 78,80</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>▼ 63,2%</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N87" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O87" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
           <t>01/04/2026</t>
         </is>
       </c>
-      <c r="B85" s="2" t="inlineStr">
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>3076915307</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>R$ 77,90</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>R$ 952,00</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr">
+        <is>
+          <t>▲ 210,1%</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="J88" s="4" t="inlineStr">
+        <is>
+          <t>▲ 1,2%</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>15,5%</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>11,3%</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>6311164080</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>R$ 78,80</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>▼ 26,9%</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O89" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>31/03/2026</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>BRINQ-019</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr">
-        <is>
-          <t>Vassoura infantil unicornio</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="inlineStr">
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>3076915307</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>R$ 77,90</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>R$ 307,00</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>4,8%</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>3,3%</t>
+        </is>
+      </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>31/03/2026</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
         <is>
           <t>6311164080</t>
         </is>
       </c>
-      <c r="F85" s="2" t="inlineStr">
+      <c r="F91" s="2" t="inlineStr">
         <is>
           <t>R$ 78,80</t>
         </is>
       </c>
-      <c r="G85" s="2" t="inlineStr">
+      <c r="G91" s="2" t="inlineStr">
         <is>
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H85" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I85" s="2" t="n">
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="J85" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K85" s="2" t="inlineStr">
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
         <is>
           <t>0,0%</t>
         </is>
       </c>
-      <c r="L85" s="2" t="n">
+      <c r="L91" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M85" s="2" t="inlineStr">
+      <c r="M91" s="2" t="inlineStr">
         <is>
           <t>0,0%</t>
         </is>
       </c>
-      <c r="N85" s="2" t="inlineStr">
+      <c r="N91" s="2" t="inlineStr">
         <is>
           <t>Sem calcular</t>
         </is>
       </c>
-      <c r="O85" s="2" t="inlineStr">
+      <c r="O91" s="2" t="inlineStr">
         <is>
           <t>Boa</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O85"/>
+  <autoFilter ref="A1:O91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
relatorio 15-05 | 16-05 | 17-05
</commit_message>
<xml_diff>
--- a/saida_skus/SKU_BRINQ-019-VASSOURA-INFANTIL-UNICORNIO.xlsx
+++ b/saida_skus/SKU_BRINQ-019-VASSOURA-INFANTIL-UNICORNIO.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Analise" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analise'!$A$1:$O$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analise'!$A$1:$O$97</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O91"/>
+  <dimension ref="A1:O97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -559,12 +559,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>15/05/2026</t>
+          <t>18/05/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>14/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -632,12 +632,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>15/05/2026</t>
+          <t>18/05/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>14/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -709,12 +709,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>14/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -747,10 +747,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I4" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -759,39 +757,37 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Boa</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>14/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -863,12 +859,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>12/05/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -936,12 +932,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>12/05/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1013,12 +1009,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>12/05/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>14/05/2026</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1086,12 +1082,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>12/05/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>14/05/2026</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1163,12 +1159,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>14/05/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>10/05/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1193,7 +1189,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1201,8 +1197,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I10" s="2" t="n">
-        <v>0</v>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -1211,37 +1209,39 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>14/05/2026</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>10/05/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1313,12 +1313,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>10/05/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>12/05/2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1351,10 +1351,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I12" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
@@ -1363,39 +1361,37 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Boa</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>10/05/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>12/05/2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1467,12 +1463,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>12/05/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1497,7 +1493,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1505,10 +1501,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I14" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
@@ -1517,39 +1511,37 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Boa</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>12/05/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1621,12 +1613,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1694,12 +1686,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1771,12 +1763,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1801,7 +1793,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1809,8 +1801,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I18" s="2" t="n">
-        <v>0</v>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
@@ -1819,37 +1813,39 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1921,12 +1917,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1951,7 +1947,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1959,8 +1955,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I20" s="2" t="n">
-        <v>0</v>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
@@ -1969,37 +1967,39 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2071,12 +2071,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2112,9 +2112,9 @@
       <c r="I22" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -2144,12 +2144,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2221,12 +2221,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2260,7 +2260,7 @@
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
@@ -2294,12 +2294,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2371,12 +2371,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2412,9 +2412,9 @@
       <c r="I26" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J26" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2444,12 +2444,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2521,12 +2521,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2560,11 +2560,11 @@
         </is>
       </c>
       <c r="I28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>0</v>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2594,12 +2594,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2671,12 +2671,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2710,7 +2710,7 @@
         </is>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
@@ -2744,12 +2744,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2821,12 +2821,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2862,9 +2862,9 @@
       <c r="I32" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -2894,12 +2894,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2971,12 +2971,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -3009,10 +3009,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I34" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
@@ -3021,39 +3019,37 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Boa</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -3125,12 +3121,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3198,12 +3194,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3275,12 +3271,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -3348,12 +3344,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -3425,12 +3421,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -3455,7 +3451,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -3463,47 +3459,51 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J40" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L40" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -3575,12 +3575,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -3614,7 +3614,7 @@
         </is>
       </c>
       <c r="I42" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
@@ -3648,12 +3648,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -3725,12 +3725,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -3758,17 +3758,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H44" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I44" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -3798,12 +3798,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3875,12 +3875,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3905,7 +3905,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>R$ 78,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -3914,24 +3914,24 @@
         </is>
       </c>
       <c r="I46" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>0</v>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>14,3%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L46" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>1,1%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
@@ -3948,12 +3948,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -4025,12 +4025,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -4058,17 +4058,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H48" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -4098,12 +4098,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -4175,12 +4175,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -4205,33 +4205,33 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>R$ 78,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>▼ 75,0%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I50" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>0</v>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>6,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L50" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>1,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
@@ -4248,12 +4248,12 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -4325,12 +4325,12 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -4355,33 +4355,33 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>R$ 312,00</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="inlineStr">
-        <is>
-          <t>▼ 20,0%</t>
+          <t>R$ 78,00</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J52" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>7</v>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>14,3%</t>
         </is>
       </c>
       <c r="L52" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>4,0%</t>
+          <t>1,1%</t>
         </is>
       </c>
       <c r="N52" s="2" t="inlineStr">
@@ -4398,12 +4398,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -4475,12 +4475,12 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -4505,33 +4505,33 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>R$ 390,00</t>
-        </is>
-      </c>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>▲ 66,7%</t>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I54" s="2" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>▼ 4,6%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>8,1%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L54" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>5,2%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N54" s="2" t="inlineStr">
@@ -4548,12 +4548,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -4625,12 +4625,12 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -4655,33 +4655,33 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>R$ 234,00</t>
+          <t>R$ 78,00</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>▼ 49,9%</t>
+          <t>▼ 75,0%</t>
         </is>
       </c>
       <c r="I56" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="J56" s="3" t="inlineStr">
-        <is>
-          <t>▼ 28,6%</t>
+        <v>15</v>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>4,6%</t>
+          <t>6,7%</t>
         </is>
       </c>
       <c r="L56" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>3,6%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N56" s="2" t="inlineStr">
@@ -4698,12 +4698,12 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -4775,12 +4775,12 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -4805,33 +4805,33 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>R$ 467,00</t>
-        </is>
-      </c>
-      <c r="H58" s="4" t="inlineStr">
-        <is>
-          <t>▲ 199,4%</t>
+          <t>R$ 312,00</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>▼ 20,0%</t>
         </is>
       </c>
       <c r="I58" s="2" t="n">
-        <v>91</v>
-      </c>
-      <c r="J58" s="4" t="inlineStr">
-        <is>
-          <t>▲ 49,2%</t>
+        <v>0</v>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>6,6%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L58" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>4,7%</t>
+          <t>4,0%</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr">
@@ -4848,12 +4848,12 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -4925,12 +4925,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -4955,33 +4955,33 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>R$ 156,00</t>
-        </is>
-      </c>
-      <c r="H60" s="3" t="inlineStr">
-        <is>
-          <t>▼ 33,3%</t>
+          <t>R$ 390,00</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>▲ 66,7%</t>
         </is>
       </c>
       <c r="I60" s="2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>▼ 19,7%</t>
+          <t>▼ 4,6%</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>3,3%</t>
+          <t>8,1%</t>
         </is>
       </c>
       <c r="L60" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>1,7%</t>
+          <t>5,2%</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
@@ -4998,12 +4998,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -5075,12 +5075,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -5114,16 +5114,16 @@
         </is>
       </c>
       <c r="I62" s="2" t="n">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>▼ 2,6%</t>
+          <t>▼ 28,6%</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>3,9%</t>
+          <t>4,6%</t>
         </is>
       </c>
       <c r="L62" s="2" t="n">
@@ -5131,7 +5131,7 @@
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>2,1%</t>
+          <t>3,6%</t>
         </is>
       </c>
       <c r="N62" s="2" t="inlineStr">
@@ -5148,12 +5148,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -5225,12 +5225,12 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -5258,22 +5258,22 @@
           <t>R$ 467,00</t>
         </is>
       </c>
-      <c r="H64" s="3" t="inlineStr">
-        <is>
-          <t>▼ 14,3%</t>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>▲ 199,4%</t>
         </is>
       </c>
       <c r="I64" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="J64" s="3" t="inlineStr">
-        <is>
-          <t>▼ 27,1%</t>
+        <v>91</v>
+      </c>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>▲ 49,2%</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>7,7%</t>
+          <t>6,6%</t>
         </is>
       </c>
       <c r="L64" s="2" t="n">
@@ -5281,7 +5281,7 @@
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>4,3%</t>
+          <t>4,7%</t>
         </is>
       </c>
       <c r="N64" s="2" t="inlineStr">
@@ -5298,12 +5298,12 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -5375,12 +5375,12 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -5405,33 +5405,33 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>R$ 545,00</t>
-        </is>
-      </c>
-      <c r="H66" s="4" t="inlineStr">
-        <is>
-          <t>▲ 74,7%</t>
+          <t>R$ 156,00</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>▼ 33,3%</t>
         </is>
       </c>
       <c r="I66" s="2" t="n">
-        <v>107</v>
-      </c>
-      <c r="J66" s="4" t="inlineStr">
-        <is>
-          <t>▲ 10,3%</t>
+        <v>61</v>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>▼ 19,7%</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>6,5%</t>
+          <t>3,3%</t>
         </is>
       </c>
       <c r="L66" s="2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>4,5%</t>
+          <t>1,7%</t>
         </is>
       </c>
       <c r="N66" s="2" t="inlineStr">
@@ -5448,12 +5448,12 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -5478,7 +5478,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -5486,8 +5486,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I67" s="2" t="n">
-        <v>0</v>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
@@ -5496,37 +5498,39 @@
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L67" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N67" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -5551,33 +5555,33 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>R$ 312,00</t>
-        </is>
-      </c>
-      <c r="H68" s="4" t="inlineStr">
-        <is>
-          <t>▲ 300,0%</t>
+          <t>R$ 234,00</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>▼ 49,9%</t>
         </is>
       </c>
       <c r="I68" s="2" t="n">
-        <v>97</v>
-      </c>
-      <c r="J68" s="4" t="inlineStr">
-        <is>
-          <t>▲ 203,1%</t>
+        <v>76</v>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>▼ 2,6%</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>4,1%</t>
+          <t>3,9%</t>
         </is>
       </c>
       <c r="L68" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>4,7%</t>
+          <t>2,1%</t>
         </is>
       </c>
       <c r="N68" s="2" t="inlineStr">
@@ -5594,12 +5598,12 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -5624,7 +5628,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -5632,8 +5636,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I69" s="2" t="n">
-        <v>0</v>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
@@ -5642,37 +5648,39 @@
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L69" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M69" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N69" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -5697,38 +5705,38 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>R$ 78,00</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 467,00</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>▼ 14,3%</t>
         </is>
       </c>
       <c r="I70" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="J70" s="4" t="inlineStr">
-        <is>
-          <t>▲ 1500,0%</t>
+        <v>78</v>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>▼ 27,1%</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>3,1%</t>
+          <t>7,7%</t>
         </is>
       </c>
       <c r="L70" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M70" s="2" t="inlineStr">
         <is>
-          <t>1,0%</t>
+          <t>4,3%</t>
         </is>
       </c>
       <c r="N70" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O70" s="2" t="inlineStr">
@@ -5740,12 +5748,12 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -5770,7 +5778,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -5778,47 +5786,51 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I71" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J71" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L71" s="2" t="n">
-        <v>0</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N71" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -5843,33 +5855,33 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 545,00</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>▲ 74,7%</t>
         </is>
       </c>
       <c r="I72" s="2" t="n">
-        <v>2</v>
+        <v>107</v>
       </c>
       <c r="J72" s="4" t="inlineStr">
         <is>
-          <t>▲ 100,0%</t>
+          <t>▲ 10,3%</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>6,5%</t>
         </is>
       </c>
       <c r="L72" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>4,5%</t>
         </is>
       </c>
       <c r="N72" s="2" t="inlineStr">
@@ -5886,12 +5898,12 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -5919,17 +5931,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H73" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I73" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="J73" s="4" t="inlineStr">
-        <is>
-          <t>▲ 200,0%</t>
+        <v>0</v>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -5959,12 +5971,12 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -5989,33 +6001,33 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
-        </is>
-      </c>
-      <c r="H74" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+          <t>R$ 312,00</t>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>▲ 300,0%</t>
         </is>
       </c>
       <c r="I74" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J74" s="3" t="inlineStr">
-        <is>
-          <t>▼ 99,2%</t>
+        <v>97</v>
+      </c>
+      <c r="J74" s="4" t="inlineStr">
+        <is>
+          <t>▲ 203,1%</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>4,1%</t>
         </is>
       </c>
       <c r="L74" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>4,7%</t>
         </is>
       </c>
       <c r="N74" s="2" t="inlineStr">
@@ -6032,12 +6044,12 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -6062,7 +6074,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>R$ 75,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -6071,7 +6083,7 @@
         </is>
       </c>
       <c r="I75" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
@@ -6080,15 +6092,15 @@
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>50,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L75" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>1,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N75" s="2" t="inlineStr">
@@ -6105,12 +6117,12 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -6135,38 +6147,38 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>R$ 659,00</t>
-        </is>
-      </c>
-      <c r="H76" s="4" t="inlineStr">
-        <is>
-          <t>▲ 124,9%</t>
+          <t>R$ 78,00</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I76" s="2" t="n">
-        <v>120</v>
+        <v>32</v>
       </c>
       <c r="J76" s="4" t="inlineStr">
         <is>
-          <t>▲ 4,3%</t>
+          <t>▲ 1500,0%</t>
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>7,5%</t>
+          <t>3,1%</t>
         </is>
       </c>
       <c r="L76" s="2" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>6,5%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N76" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Sem calcular</t>
         </is>
       </c>
       <c r="O76" s="2" t="inlineStr">
@@ -6178,12 +6190,12 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -6211,9 +6223,9 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H77" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I77" s="2" t="n">
@@ -6251,12 +6263,12 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -6281,38 +6293,38 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>R$ 293,00</t>
-        </is>
-      </c>
-      <c r="H78" s="3" t="inlineStr">
-        <is>
-          <t>▼ 33,3%</t>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I78" s="2" t="n">
-        <v>115</v>
-      </c>
-      <c r="J78" s="3" t="inlineStr">
-        <is>
-          <t>▼ 12,2%</t>
+        <v>2</v>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>3,5%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L78" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M78" s="2" t="inlineStr">
         <is>
-          <t>2,8%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N78" s="2" t="inlineStr">
         <is>
-          <t>Sem calcular</t>
+          <t>Básica</t>
         </is>
       </c>
       <c r="O78" s="2" t="inlineStr">
@@ -6324,12 +6336,12 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -6354,33 +6366,33 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>R$ 75,00</t>
-        </is>
-      </c>
-      <c r="H79" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I79" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="J79" s="3" t="inlineStr">
-        <is>
-          <t>▼ 12,5%</t>
+        <v>6</v>
+      </c>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>▲ 200,0%</t>
         </is>
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>14,3%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L79" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M79" s="2" t="inlineStr">
         <is>
-          <t>0,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N79" s="2" t="inlineStr">
@@ -6397,12 +6409,12 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -6427,33 +6439,33 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>R$ 439,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>▼ 25,1%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I80" s="2" t="n">
-        <v>131</v>
+        <v>1</v>
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>▼ 0,8%</t>
+          <t>▼ 99,2%</t>
         </is>
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>4,6%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L80" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M80" s="2" t="inlineStr">
         <is>
-          <t>4,8%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N80" s="2" t="inlineStr">
@@ -6470,12 +6482,12 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -6500,7 +6512,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 75,00</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -6509,24 +6521,24 @@
         </is>
       </c>
       <c r="I81" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="J81" s="3" t="inlineStr">
-        <is>
-          <t>▼ 20,0%</t>
+        <v>2</v>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>50,0%</t>
         </is>
       </c>
       <c r="L81" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M81" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>1,0%</t>
         </is>
       </c>
       <c r="N81" s="2" t="inlineStr">
@@ -6543,12 +6555,12 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -6573,33 +6585,33 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>R$ 586,00</t>
-        </is>
-      </c>
-      <c r="H82" s="3" t="inlineStr">
-        <is>
-          <t>▼ 11,1%</t>
+          <t>R$ 659,00</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>▲ 124,9%</t>
         </is>
       </c>
       <c r="I82" s="2" t="n">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J82" s="4" t="inlineStr">
         <is>
-          <t>▲ 34,7%</t>
+          <t>▲ 4,3%</t>
         </is>
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>6,1%</t>
+          <t>7,5%</t>
         </is>
       </c>
       <c r="L82" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M82" s="2" t="inlineStr">
         <is>
-          <t>6,8%</t>
+          <t>6,5%</t>
         </is>
       </c>
       <c r="N82" s="2" t="inlineStr">
@@ -6616,12 +6628,12 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -6655,11 +6667,11 @@
         </is>
       </c>
       <c r="I83" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J83" s="4" t="inlineStr">
-        <is>
-          <t>▲ 25,0%</t>
+        <v>0</v>
+      </c>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K83" s="2" t="inlineStr">
@@ -6689,12 +6701,12 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -6719,38 +6731,38 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>R$ 659,00</t>
-        </is>
-      </c>
-      <c r="H84" s="4" t="inlineStr">
-        <is>
-          <t>▲ 80,1%</t>
+          <t>R$ 293,00</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>▼ 33,3%</t>
         </is>
       </c>
       <c r="I84" s="2" t="n">
-        <v>98</v>
-      </c>
-      <c r="J84" s="4" t="inlineStr">
-        <is>
-          <t>▲ 3,2%</t>
+        <v>115</v>
+      </c>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>▼ 12,2%</t>
         </is>
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t>9,2%</t>
+          <t>3,5%</t>
         </is>
       </c>
       <c r="L84" s="2" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="M84" s="2" t="inlineStr">
         <is>
-          <t>6,3%</t>
+          <t>2,8%</t>
         </is>
       </c>
       <c r="N84" s="2" t="inlineStr">
         <is>
-          <t>Básica</t>
+          <t>Sem calcular</t>
         </is>
       </c>
       <c r="O84" s="2" t="inlineStr">
@@ -6762,12 +6774,12 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
@@ -6801,16 +6813,16 @@
         </is>
       </c>
       <c r="I85" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="J85" s="4" t="inlineStr">
-        <is>
-          <t>▲ 14,3%</t>
+        <v>7</v>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>▼ 12,5%</t>
         </is>
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
-          <t>12,5%</t>
+          <t>14,3%</t>
         </is>
       </c>
       <c r="L85" s="2" t="n">
@@ -6835,12 +6847,12 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -6865,29 +6877,29 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>R$ 366,00</t>
+          <t>R$ 439,00</t>
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>▼ 61,6%</t>
+          <t>▼ 25,1%</t>
         </is>
       </c>
       <c r="I86" s="2" t="n">
-        <v>95</v>
-      </c>
-      <c r="J86" s="4" t="inlineStr">
-        <is>
-          <t>▲ 13,1%</t>
+        <v>131</v>
+      </c>
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t>▼ 0,8%</t>
         </is>
       </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
-          <t>5,3%</t>
+          <t>4,6%</t>
         </is>
       </c>
       <c r="L86" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M86" s="2" t="inlineStr">
         <is>
@@ -6908,12 +6920,12 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -6947,11 +6959,11 @@
         </is>
       </c>
       <c r="I87" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>▼ 63,2%</t>
+          <t>▼ 20,0%</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
@@ -6981,12 +6993,12 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -7011,33 +7023,33 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>R$ 952,00</t>
-        </is>
-      </c>
-      <c r="H88" s="4" t="inlineStr">
-        <is>
-          <t>▲ 210,1%</t>
+          <t>R$ 586,00</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>▼ 11,1%</t>
         </is>
       </c>
       <c r="I88" s="2" t="n">
-        <v>84</v>
+        <v>132</v>
       </c>
       <c r="J88" s="4" t="inlineStr">
         <is>
-          <t>▲ 1,2%</t>
+          <t>▲ 34,7%</t>
         </is>
       </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t>15,5%</t>
+          <t>6,1%</t>
         </is>
       </c>
       <c r="L88" s="2" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="M88" s="2" t="inlineStr">
         <is>
-          <t>11,3%</t>
+          <t>6,8%</t>
         </is>
       </c>
       <c r="N88" s="2" t="inlineStr">
@@ -7054,12 +7066,12 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -7087,17 +7099,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H89" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I89" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="J89" s="3" t="inlineStr">
-        <is>
-          <t>▼ 26,9%</t>
+        <v>10</v>
+      </c>
+      <c r="J89" s="4" t="inlineStr">
+        <is>
+          <t>▲ 25,0%</t>
         </is>
       </c>
       <c r="K89" s="2" t="inlineStr">
@@ -7127,12 +7139,12 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>03/04/2026</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -7157,33 +7169,33 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>R$ 307,00</t>
-        </is>
-      </c>
-      <c r="H90" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>R$ 659,00</t>
+        </is>
+      </c>
+      <c r="H90" s="4" t="inlineStr">
+        <is>
+          <t>▲ 80,1%</t>
         </is>
       </c>
       <c r="I90" s="2" t="n">
-        <v>83</v>
-      </c>
-      <c r="J90" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>98</v>
+      </c>
+      <c r="J90" s="4" t="inlineStr">
+        <is>
+          <t>▲ 3,2%</t>
         </is>
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
-          <t>4,8%</t>
+          <t>9,2%</t>
         </is>
       </c>
       <c r="L90" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="M90" s="2" t="inlineStr">
         <is>
-          <t>3,3%</t>
+          <t>6,3%</t>
         </is>
       </c>
       <c r="N90" s="2" t="inlineStr">
@@ -7200,78 +7212,516 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
+          <t>04/04/2026</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>6311164080</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>R$ 78,80</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>R$ 75,00</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J91" s="4" t="inlineStr">
+        <is>
+          <t>▲ 14,3%</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>12,5%</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>0,7%</t>
+        </is>
+      </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O91" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>3076915307</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>R$ 77,90</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>R$ 366,00</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>▼ 61,6%</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="J92" s="4" t="inlineStr">
+        <is>
+          <t>▲ 13,1%</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>5,3%</t>
+        </is>
+      </c>
+      <c r="L92" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>4,8%</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>6311164080</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>R$ 78,80</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J93" s="3" t="inlineStr">
+        <is>
+          <t>▼ 63,2%</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N93" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O93" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
           <t>01/04/2026</t>
         </is>
       </c>
-      <c r="B91" s="2" t="inlineStr">
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>3076915307</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>R$ 77,90</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>R$ 952,00</t>
+        </is>
+      </c>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>▲ 210,1%</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="J94" s="4" t="inlineStr">
+        <is>
+          <t>▲ 1,2%</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>15,5%</t>
+        </is>
+      </c>
+      <c r="L94" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>11,3%</t>
+        </is>
+      </c>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>6311164080</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>R$ 78,80</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="J95" s="3" t="inlineStr">
+        <is>
+          <t>▼ 26,9%</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N95" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O95" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
         <is>
           <t>31/03/2026</t>
         </is>
       </c>
-      <c r="C91" s="2" t="inlineStr">
-        <is>
-          <t>BRINQ-019</t>
-        </is>
-      </c>
-      <c r="D91" s="2" t="inlineStr">
-        <is>
-          <t>Vassoura infantil unicornio</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>3076915307</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>R$ 77,90</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>R$ 307,00</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>4,8%</t>
+        </is>
+      </c>
+      <c r="L96" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>3,3%</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>Básica</t>
+        </is>
+      </c>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>31/03/2026</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>BRINQ-019</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Vassoura infantil unicornio</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
         <is>
           <t>6311164080</t>
         </is>
       </c>
-      <c r="F91" s="2" t="inlineStr">
+      <c r="F97" s="2" t="inlineStr">
         <is>
           <t>R$ 78,80</t>
         </is>
       </c>
-      <c r="G91" s="2" t="inlineStr">
+      <c r="G97" s="2" t="inlineStr">
         <is>
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H91" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I91" s="2" t="n">
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="J91" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K91" s="2" t="inlineStr">
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr">
         <is>
           <t>0,0%</t>
         </is>
       </c>
-      <c r="L91" s="2" t="n">
+      <c r="L97" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M91" s="2" t="inlineStr">
+      <c r="M97" s="2" t="inlineStr">
         <is>
           <t>0,0%</t>
         </is>
       </c>
-      <c r="N91" s="2" t="inlineStr">
+      <c r="N97" s="2" t="inlineStr">
         <is>
           <t>Sem calcular</t>
         </is>
       </c>
-      <c r="O91" s="2" t="inlineStr">
+      <c r="O97" s="2" t="inlineStr">
         <is>
           <t>Boa</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O91"/>
+  <autoFilter ref="A1:O97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>